<commit_message>
fix: preserve workbook compatibility and existing authoring permissions
</commit_message>
<xml_diff>
--- a/src/ClimateProject.Api/Assets/TIMS_NEXA_Clima_Integral.xlsx
+++ b/src/ClimateProject.Api/Assets/TIMS_NEXA_Clima_Integral.xlsx
@@ -695,7 +695,7 @@
     <xdr:ext cx="1295400" cy="666750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="c266e7f9-979e-4fae-9aa9-62fcd1de6bd9"/>
+        <xdr:cNvPr id="1" name="Brand image 1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -722,7 +722,7 @@
     <xdr:ext cx="609600" cy="609600"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="3ec50c4e-47f6-4697-8353-39e786e40e84"/>
+        <xdr:cNvPr id="2" name="Brand image 2"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -754,7 +754,7 @@
     <xdr:ext cx="1295400" cy="666750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="ed05cd19-e6f8-46df-a1fe-4bfff80fd6d9"/>
+        <xdr:cNvPr id="1" name="Brand image 1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -781,7 +781,7 @@
     <xdr:ext cx="609600" cy="609600"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="a4d1a03e-c136-4b61-b4ed-b6616669a6e3"/>
+        <xdr:cNvPr id="2" name="Brand image 2"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -813,7 +813,7 @@
     <xdr:ext cx="1295400" cy="666750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="014f9ebb-e78c-41bc-bcc2-e893e71187a7"/>
+        <xdr:cNvPr id="1" name="Brand image 1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -840,7 +840,7 @@
     <xdr:ext cx="609600" cy="609600"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="2dc1a4a5-bc4e-4566-864a-0264931428f2"/>
+        <xdr:cNvPr id="2" name="Brand image 2"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -872,7 +872,7 @@
     <xdr:ext cx="1295400" cy="666750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="b4148e7f-821b-44d1-ae0e-fbbd2e873597"/>
+        <xdr:cNvPr id="1" name="Brand image 1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -899,7 +899,7 @@
     <xdr:ext cx="609600" cy="609600"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="854e1100-102c-4037-9e42-ea5877505557"/>
+        <xdr:cNvPr id="2" name="Brand image 2"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -931,7 +931,7 @@
     <xdr:ext cx="1295400" cy="666750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="2db593fa-5dbc-49e2-996e-c8414faeecd0"/>
+        <xdr:cNvPr id="1" name="Brand image 1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -958,7 +958,7 @@
     <xdr:ext cx="609600" cy="609600"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="c4cd30f6-7037-4e60-9221-97dab5a2e269"/>
+        <xdr:cNvPr id="2" name="Brand image 2"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -990,7 +990,7 @@
     <xdr:ext cx="1295400" cy="666750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="3a0682bc-84a0-434b-bc03-380b922ee728"/>
+        <xdr:cNvPr id="1" name="Brand image 1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1017,7 +1017,7 @@
     <xdr:ext cx="609600" cy="609600"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="13ba7014-cc5f-4946-96c7-ceb3b8f8a659"/>
+        <xdr:cNvPr id="2" name="Brand image 2"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1049,7 +1049,7 @@
     <xdr:ext cx="1295400" cy="666750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1a0d273c-1119-4c9d-872a-6592d2aa8cef"/>
+        <xdr:cNvPr id="1" name="Brand image 1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1076,7 +1076,7 @@
     <xdr:ext cx="609600" cy="609600"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="82830e76-29b9-4019-99c8-e7daebc0adf1"/>
+        <xdr:cNvPr id="2" name="Brand image 2"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>

</xml_diff>